<commit_message>
Finalize FinSight submission package
</commit_message>
<xml_diff>
--- a/sample_data/FinSight_Test_Data_Catalog.xlsx
+++ b/sample_data/FinSight_Test_Data_Catalog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upload Test Catalog" sheetId="1" r:id="R2b4728bea2944d07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upload Test Catalog" sheetId="1" r:id="Rfb07d62a15a149ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -572,7 +572,7 @@
         <x:v>Leave missing fields unmapped</x:v>
       </x:c>
       <x:c r="F7" s="33" t="str">
-        <x:v>What should we measure for onboarding?</x:v>
+        <x:v>How are customers progressing from card activation to first transaction and 30-day activity?</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">

</xml_diff>